<commit_message>
T3 fix: DAILY vao xlsx, xoa CSV, cap nhat CLAUDE.md
- CASE_TAG.xlsx DAILY row 31: them 29/07 (O=1.6204, P=1.3719, Q=1.8129 fn=1 SUSPECT)
- CASE_BR.xlsx DAILY row 67: them G/H/I f_min/max/n (khong de chong data operator)
- Xoa TAG_daily.csv + BR_daily.csv khoi git (an 30/07: DAILY song trong xlsx, khong CSV)
- CLAUDE.md: them quy tac cam sinh CSV trong docs/case_files/ (an 30/07, tai pham 1 lan)
- .gitignore: revert exception khong can nua

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_TAG.xlsx
+++ b/docs/case_files/CASE_TAG.xlsx
@@ -639,12 +639,12 @@
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="29">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="28" t="inlineStr">
         <is>
           <t>LEGEND</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="28" t="inlineStr">
         <is>
           <t>oi_vs_med14 Excel != dinh nghia fire — window ending khac signals.py (signals.py dung window ket thuc ngay-truoc-check; DAILY dung window khac, chi nhin nhanh)</t>
         </is>
@@ -3227,6 +3227,86 @@
         <v/>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="C31">
+        <f>IFERROR(B31/B30-1,"")</f>
+        <v/>
+      </c>
+      <c r="F31" t="n">
+        <v>0.00014019</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0.00014019</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0.00014019</v>
+      </c>
+      <c r="I31" t="n">
+        <v>1</v>
+      </c>
+      <c r="J31" t="inlineStr"/>
+      <c r="L31" t="n">
+        <v>11172261</v>
+      </c>
+      <c r="M31">
+        <f>IFERROR(L31/MEDIAN(L17:L30),"")</f>
+        <v/>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>PEAK</t>
+        </is>
+      </c>
+      <c r="O31" t="n">
+        <v>1.6204</v>
+      </c>
+      <c r="P31" t="n">
+        <v>1.3719</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>1.8129</v>
+      </c>
+      <c r="R31">
+        <f>IFERROR(O31/P31,"")</f>
+        <v/>
+      </c>
+      <c r="S31">
+        <f>IFERROR(AVERAGE(R29:R31),"")</f>
+        <v/>
+      </c>
+      <c r="T31">
+        <f>IFERROR(Q31/Q26,"")</f>
+        <v/>
+      </c>
+      <c r="U31">
+        <f>IFERROR(O31/O28-1,"")</f>
+        <v/>
+      </c>
+      <c r="V31">
+        <f>IFERROR(P31/P28-1,"")</f>
+        <v/>
+      </c>
+      <c r="Z31" t="inlineStr"/>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>gate</t>
+        </is>
+      </c>
+      <c r="AJ31">
+        <f>IF(OR(AB31="",D31="",D31=0),"",AB31/D31)</f>
+        <v/>
+      </c>
+      <c r="AN31" t="inlineStr">
+        <is>
+          <t>gLSR 1.8129 fn=1 low_conf — single snapshot, suspect spike; acc_r 0.999-&gt;1.372 keo div_raw 1.597-&gt;1.181</t>
+        </is>
+      </c>
+    </row>
     <row r="32" ht="15" customHeight="1" s="29">
       <c r="A32" s="36" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
TAG chốt canh T1-T6 + DAILY fix 30/07 + append 01-03/08 (04/08)
- Probe T1-T6: chuỗi 28/07→03/08 đầy đủ — 4h funding cycle xác nhận
- INVALIDATE: lần đầu bắn 29/07 (ret_3d=+8.6%, gLSR=1.81); tiếp 31/07-02/08; ngưng 03/08
- gLSR 03/08 = 2.067 (cao nhất); crowd flush MAX -19.7% (thiếu -30% L-26)
- Exit cờ: 2/5 (③01/08 funding burst, ⑤31/07 px+/OI-)
- CASE_TAG.xlsx DAILY: unmerge A32:L32, ghi 30/07 px=0.001099 OI=9.66M; append 01-03/08

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_TAG.xlsx
+++ b/docs/case_files/CASE_TAG.xlsx
@@ -803,7 +803,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AO33"/>
+  <dimension ref="A1:AO36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="28" min="1" max="1"/>
@@ -3318,6 +3318,39 @@
           <t>2026-07-30</t>
         </is>
       </c>
+      <c r="B32" t="n">
+        <v>0.0010992966649597</v>
+      </c>
+      <c r="C32">
+        <f>IFERROR(B32/B31-1,"")</f>
+        <v/>
+      </c>
+      <c r="D32" t="n">
+        <v>3484443.358583</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0.4908091043332145</v>
+      </c>
+      <c r="F32" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="G32" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="H32" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="I32" t="n">
+        <v>6</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>PINNED</t>
+        </is>
+      </c>
+      <c r="L32" t="n">
+        <v>9658576.732218999</v>
+      </c>
       <c r="O32" s="28" t="n">
         <v>1.6632</v>
       </c>
@@ -3353,79 +3386,287 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="28" t="inlineStr">
         <is>
           <t>2026-07-31</t>
         </is>
       </c>
-      <c r="B33" t="n">
+      <c r="B33" s="28" t="n">
         <v>0.001355734069612156</v>
       </c>
-      <c r="C33">
+      <c r="C33" s="28">
         <f>IFERROR(B33/B32-1,"")</f>
         <v/>
       </c>
-      <c r="D33" t="n">
+      <c r="D33" s="28" t="n">
         <v>20833007.401828</v>
       </c>
-      <c r="E33" t="n">
+      <c r="E33" s="28" t="n">
         <v>0.5010726937085267</v>
       </c>
-      <c r="F33" t="n">
+      <c r="F33" s="28" t="n">
         <v>0.0001649366666666667</v>
       </c>
-      <c r="G33" t="n">
-        <v>5e-05</v>
-      </c>
-      <c r="H33" t="n">
+      <c r="G33" s="28" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="H33" s="28" t="n">
         <v>0.00046994</v>
       </c>
-      <c r="I33" t="n">
+      <c r="I33" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="L33" t="n">
+      <c r="L33" s="28" t="n">
         <v>9375186.135129569</v>
       </c>
-      <c r="O33" t="n">
+      <c r="O33" s="28" t="n">
         <v>1.6811</v>
       </c>
-      <c r="P33" t="n">
+      <c r="P33" s="28" t="n">
         <v>1.4795</v>
       </c>
-      <c r="Q33" t="n">
+      <c r="Q33" s="28" t="n">
         <v>1.9223</v>
       </c>
-      <c r="R33">
+      <c r="R33" s="28">
         <f>IFERROR(O33/P33,"")</f>
         <v/>
       </c>
-      <c r="S33">
+      <c r="S33" s="28">
         <f>IFERROR(AVERAGE(R31:R33),"")</f>
         <v/>
       </c>
-      <c r="T33">
+      <c r="T33" s="28">
         <f>IFERROR(Q33/Q28,"")</f>
         <v/>
       </c>
-      <c r="U33">
+      <c r="U33" s="28">
         <f>IFERROR(O33/O30-1,"")</f>
         <v/>
       </c>
-      <c r="V33">
+      <c r="V33" s="28">
         <f>IFERROR(P33/P30-1,"")</f>
         <v/>
       </c>
-      <c r="AJ33">
+      <c r="AJ33" s="28">
         <f>IF(OR(AB33="",D33="",D33=0),"",AB33/D33)</f>
         <v/>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>0.001387312420744</v>
+      </c>
+      <c r="C34">
+        <f>IFERROR(B34/B33-1,"")</f>
+        <v/>
+      </c>
+      <c r="D34" t="n">
+        <v>14173987.853918</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0.5132635677780482</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0.0002554233333333</v>
+      </c>
+      <c r="G34" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0.00056037</v>
+      </c>
+      <c r="I34" t="n">
+        <v>6</v>
+      </c>
+      <c r="L34" t="n">
+        <v>12570735.627408</v>
+      </c>
+      <c r="M34">
+        <f>IFERROR(L34/MEDIAN(L20:L33),"")</f>
+        <v/>
+      </c>
+      <c r="O34" t="n">
+        <v>1.5905</v>
+      </c>
+      <c r="P34" t="n">
+        <v>1.2753</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>1.6157</v>
+      </c>
+      <c r="R34">
+        <f>IFERROR(O34/P34,"")</f>
+        <v/>
+      </c>
+      <c r="S34">
+        <f>IFERROR(AVERAGE(R32:R34),"")</f>
+        <v/>
+      </c>
+      <c r="T34">
+        <f>IFERROR(Q34/Q29,"")</f>
+        <v/>
+      </c>
+      <c r="U34">
+        <f>IFERROR(O34/O31-1,"")</f>
+        <v/>
+      </c>
+      <c r="V34">
+        <f>IFERROR(P34/P31-1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>0.0013870979357402</v>
+      </c>
+      <c r="C35">
+        <f>IFERROR(B35/B34-1,"")</f>
+        <v/>
+      </c>
+      <c r="D35" t="n">
+        <v>8050293.311166001</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0.4690171507460309</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0.000104545</v>
+      </c>
+      <c r="G35" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0.00027156</v>
+      </c>
+      <c r="I35" t="n">
+        <v>6</v>
+      </c>
+      <c r="L35" t="n">
+        <v>13201306.884897</v>
+      </c>
+      <c r="M35">
+        <f>IFERROR(L35/MEDIAN(L21:L34),"")</f>
+        <v/>
+      </c>
+      <c r="O35" t="n">
+        <v>1.2863</v>
+      </c>
+      <c r="P35" t="n">
+        <v>1.5981</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>1.956</v>
+      </c>
+      <c r="R35">
+        <f>IFERROR(O35/P35,"")</f>
+        <v/>
+      </c>
+      <c r="S35">
+        <f>IFERROR(AVERAGE(R33:R35),"")</f>
+        <v/>
+      </c>
+      <c r="T35">
+        <f>IFERROR(Q35/Q30,"")</f>
+        <v/>
+      </c>
+      <c r="U35">
+        <f>IFERROR(O35/O32-1,"")</f>
+        <v/>
+      </c>
+      <c r="V35">
+        <f>IFERROR(P35/P32-1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>0.001259841794361022</v>
+      </c>
+      <c r="C36">
+        <f>IFERROR(B36/B35-1,"")</f>
+        <v/>
+      </c>
+      <c r="D36" t="n">
+        <v>4779652.221457</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0.4728796584260186</v>
+      </c>
+      <c r="F36" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="G36" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="H36" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="I36" t="n">
+        <v>6</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>PINNED</t>
+        </is>
+      </c>
+      <c r="L36" t="n">
+        <v>11828955.093356</v>
+      </c>
+      <c r="M36">
+        <f>IFERROR(L36/MEDIAN(L22:L35),"")</f>
+        <v/>
+      </c>
+      <c r="O36" t="n">
+        <v>1.3504</v>
+      </c>
+      <c r="P36" t="n">
+        <v>1.7367</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>2.0665</v>
+      </c>
+      <c r="R36">
+        <f>IFERROR(O36/P36,"")</f>
+        <v/>
+      </c>
+      <c r="S36">
+        <f>IFERROR(AVERAGE(R34:R36),"")</f>
+        <v/>
+      </c>
+      <c r="T36">
+        <f>IFERROR(Q36/Q31,"")</f>
+        <v/>
+      </c>
+      <c r="U36">
+        <f>IFERROR(O36/O33-1,"")</f>
+        <v/>
+      </c>
+      <c r="V36">
+        <f>IFERROR(P36/P33-1,"")</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="4">
     <mergeCell ref="AK1:AM1"/>
     <mergeCell ref="A1:Z1"/>
     <mergeCell ref="AN1:AO1"/>
-    <mergeCell ref="A32:L32"/>
     <mergeCell ref="AA1:AJ1"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>

<commit_message>
TAG DAILY: fill spot_venue + vol_spot_usd + taker_spot_pct + alpha_suspect (04/08)
- Rows 31-36 (29/07→03/08): binance_alpha vol từ store (47K-91K USD/ngày)
- Rows 3-30 (01-28/07): giữ nguyên gate data (không overwrite)
- Tất cả: AC=ABSTAIN (taker broken trên alpha), AJ formula đầy đủ
- Alpha vol spike 08-09/07 ($479K/$668K) khớp markup start T0

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_TAG.xlsx
+++ b/docs/case_files/CASE_TAG.xlsx
@@ -1118,6 +1118,14 @@
           <t>gate</t>
         </is>
       </c>
+      <c r="AB3" t="n">
+        <v>20758.97</v>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>ABSTAIN</t>
+        </is>
+      </c>
       <c r="AJ3" s="47">
         <f>IF(OR(AB3="",D3="",D3=0),"",AB3/D3)</f>
         <v/>
@@ -1180,6 +1188,14 @@
           <t>gate</t>
         </is>
       </c>
+      <c r="AB4" t="n">
+        <v>19400.83</v>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>ABSTAIN</t>
+        </is>
+      </c>
       <c r="AJ4" s="47">
         <f>IF(OR(AB4="",D4="",D4=0),"",AB4/D4)</f>
         <v/>
@@ -1246,6 +1262,14 @@
           <t>gate</t>
         </is>
       </c>
+      <c r="AB5" t="n">
+        <v>4007.28</v>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>ABSTAIN</t>
+        </is>
+      </c>
       <c r="AJ5" s="47">
         <f>IF(OR(AB5="",D5="",D5=0),"",AB5/D5)</f>
         <v/>
@@ -1320,6 +1344,14 @@
           <t>gate</t>
         </is>
       </c>
+      <c r="AB6" t="n">
+        <v>20812.13</v>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>ABSTAIN</t>
+        </is>
+      </c>
       <c r="AJ6" s="47">
         <f>IF(OR(AB6="",D6="",D6=0),"",AB6/D6)</f>
         <v/>
@@ -1394,6 +1426,14 @@
           <t>gate</t>
         </is>
       </c>
+      <c r="AB7" t="n">
+        <v>19965.14</v>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>ABSTAIN</t>
+        </is>
+      </c>
       <c r="AJ7" s="47">
         <f>IF(OR(AB7="",D7="",D7=0),"",AB7/D7)</f>
         <v/>
@@ -1472,6 +1512,14 @@
           <t>gate</t>
         </is>
       </c>
+      <c r="AB8" t="n">
+        <v>22689.42</v>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>ABSTAIN</t>
+        </is>
+      </c>
       <c r="AJ8" s="47">
         <f>IF(OR(AB8="",D8="",D8=0),"",AB8/D8)</f>
         <v/>
@@ -1550,6 +1598,14 @@
           <t>gate</t>
         </is>
       </c>
+      <c r="AB9" t="n">
+        <v>9756.809999999999</v>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>ABSTAIN</t>
+        </is>
+      </c>
       <c r="AJ9" s="47">
         <f>IF(OR(AB9="",D9="",D9=0),"",AB9/D9)</f>
         <v/>
@@ -1628,6 +1684,14 @@
           <t>gate</t>
         </is>
       </c>
+      <c r="AB10" t="n">
+        <v>479413.99</v>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>ABSTAIN</t>
+        </is>
+      </c>
       <c r="AJ10" s="47">
         <f>IF(OR(AB10="",D10="",D10=0),"",AB10/D10)</f>
         <v/>
@@ -1711,6 +1775,14 @@
           <t>gate</t>
         </is>
       </c>
+      <c r="AB11" t="n">
+        <v>668677.45</v>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>ABSTAIN</t>
+        </is>
+      </c>
       <c r="AJ11" s="47">
         <f>IF(OR(AB11="",D11="",D11=0),"",AB11/D11)</f>
         <v/>
@@ -1794,6 +1866,14 @@
           <t>gate</t>
         </is>
       </c>
+      <c r="AB12" t="n">
+        <v>236769.36</v>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>ABSTAIN</t>
+        </is>
+      </c>
       <c r="AJ12" s="47">
         <f>IF(OR(AB12="",D12="",D12=0),"",AB12/D12)</f>
         <v/>
@@ -1872,6 +1952,14 @@
           <t>gate</t>
         </is>
       </c>
+      <c r="AB13" t="n">
+        <v>67949.34</v>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>ABSTAIN</t>
+        </is>
+      </c>
       <c r="AJ13" s="47">
         <f>IF(OR(AB13="",D13="",D13=0),"",AB13/D13)</f>
         <v/>
@@ -1950,6 +2038,14 @@
           <t>gate</t>
         </is>
       </c>
+      <c r="AB14" t="n">
+        <v>27765.15</v>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>ABSTAIN</t>
+        </is>
+      </c>
       <c r="AJ14" s="47">
         <f>IF(OR(AB14="",D14="",D14=0),"",AB14/D14)</f>
         <v/>
@@ -2028,6 +2124,14 @@
           <t>gate</t>
         </is>
       </c>
+      <c r="AB15" t="n">
+        <v>67263.77</v>
+      </c>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>ABSTAIN</t>
+        </is>
+      </c>
       <c r="AJ15" s="47">
         <f>IF(OR(AB15="",D15="",D15=0),"",AB15/D15)</f>
         <v/>
@@ -2111,6 +2215,14 @@
           <t>gate</t>
         </is>
       </c>
+      <c r="AB16" t="n">
+        <v>36889.39</v>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>ABSTAIN</t>
+        </is>
+      </c>
       <c r="AJ16" s="47">
         <f>IF(OR(AB16="",D16="",D16=0),"",AB16/D16)</f>
         <v/>
@@ -2193,6 +2305,14 @@
           <t>gate</t>
         </is>
       </c>
+      <c r="AB17" t="n">
+        <v>17499.33</v>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>ABSTAIN</t>
+        </is>
+      </c>
       <c r="AJ17" s="47">
         <f>IF(OR(AB17="",D17="",D17=0),"",AB17/D17)</f>
         <v/>
@@ -2275,6 +2395,14 @@
           <t>gate</t>
         </is>
       </c>
+      <c r="AB18" t="n">
+        <v>7085.69</v>
+      </c>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>ABSTAIN</t>
+        </is>
+      </c>
       <c r="AJ18" s="47">
         <f>IF(OR(AB18="",D18="",D18=0),"",AB18/D18)</f>
         <v/>
@@ -2362,6 +2490,14 @@
           <t>gate</t>
         </is>
       </c>
+      <c r="AB19" t="n">
+        <v>64034.17</v>
+      </c>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t>ABSTAIN</t>
+        </is>
+      </c>
       <c r="AJ19" s="47">
         <f>IF(OR(AB19="",D19="",D19=0),"",AB19/D19)</f>
         <v/>
@@ -2439,6 +2575,14 @@
           <t>gate</t>
         </is>
       </c>
+      <c r="AB20" t="n">
+        <v>49303.02</v>
+      </c>
+      <c r="AC20" t="inlineStr">
+        <is>
+          <t>ABSTAIN</t>
+        </is>
+      </c>
       <c r="AJ20" s="47">
         <f>IF(OR(AB20="",D20="",D20=0),"",AB20/D20)</f>
         <v/>
@@ -2516,6 +2660,14 @@
           <t>gate</t>
         </is>
       </c>
+      <c r="AB21" t="n">
+        <v>212614.87</v>
+      </c>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>ABSTAIN</t>
+        </is>
+      </c>
       <c r="AJ21" s="47">
         <f>IF(OR(AB21="",D21="",D21=0),"",AB21/D21)</f>
         <v/>
@@ -2593,6 +2745,14 @@
           <t>gate</t>
         </is>
       </c>
+      <c r="AB22" t="n">
+        <v>33746.04</v>
+      </c>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>ABSTAIN</t>
+        </is>
+      </c>
       <c r="AJ22" s="47">
         <f>IF(OR(AB22="",D22="",D22=0),"",AB22/D22)</f>
         <v/>
@@ -2670,6 +2830,14 @@
           <t>gate</t>
         </is>
       </c>
+      <c r="AB23" t="n">
+        <v>27282.63</v>
+      </c>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>ABSTAIN</t>
+        </is>
+      </c>
       <c r="AJ23" s="47">
         <f>IF(OR(AB23="",D23="",D23=0),"",AB23/D23)</f>
         <v/>
@@ -2747,6 +2915,14 @@
           <t>gate</t>
         </is>
       </c>
+      <c r="AB24" t="n">
+        <v>25719.93</v>
+      </c>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>ABSTAIN</t>
+        </is>
+      </c>
       <c r="AJ24" s="47">
         <f>IF(OR(AB24="",D24="",D24=0),"",AB24/D24)</f>
         <v/>
@@ -2824,6 +3000,14 @@
           <t>gate</t>
         </is>
       </c>
+      <c r="AB25" t="n">
+        <v>19137.11</v>
+      </c>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>ABSTAIN</t>
+        </is>
+      </c>
       <c r="AJ25" s="47">
         <f>IF(OR(AB25="",D25="",D25=0),"",AB25/D25)</f>
         <v/>
@@ -2901,6 +3085,14 @@
           <t>gate</t>
         </is>
       </c>
+      <c r="AB26" t="n">
+        <v>10212.63</v>
+      </c>
+      <c r="AC26" t="inlineStr">
+        <is>
+          <t>ABSTAIN</t>
+        </is>
+      </c>
       <c r="AJ26" s="47">
         <f>IF(OR(AB26="",D26="",D26=0),"",AB26/D26)</f>
         <v/>
@@ -2978,6 +3170,14 @@
           <t>gate</t>
         </is>
       </c>
+      <c r="AB27" t="n">
+        <v>4344.5</v>
+      </c>
+      <c r="AC27" t="inlineStr">
+        <is>
+          <t>ABSTAIN</t>
+        </is>
+      </c>
       <c r="AJ27" s="47">
         <f>IF(OR(AB27="",D27="",D27=0),"",AB27/D27)</f>
         <v/>
@@ -3055,6 +3255,14 @@
           <t>gate</t>
         </is>
       </c>
+      <c r="AB28" t="n">
+        <v>13320.92</v>
+      </c>
+      <c r="AC28" t="inlineStr">
+        <is>
+          <t>ABSTAIN</t>
+        </is>
+      </c>
       <c r="AJ28" s="47">
         <f>IF(OR(AB28="",D28="",D28=0),"",AB28/D28)</f>
         <v/>
@@ -3132,6 +3340,14 @@
           <t>gate</t>
         </is>
       </c>
+      <c r="AB29" t="n">
+        <v>188181.59</v>
+      </c>
+      <c r="AC29" t="inlineStr">
+        <is>
+          <t>ABSTAIN</t>
+        </is>
+      </c>
       <c r="AJ29" s="47">
         <f>IF(OR(AB29="",D29="",D29=0),"",AB29/D29)</f>
         <v/>
@@ -3226,6 +3442,11 @@
       </c>
       <c r="AB30" s="46" t="n">
         <v>33599</v>
+      </c>
+      <c r="AC30" t="inlineStr">
+        <is>
+          <t>ABSTAIN</t>
+        </is>
       </c>
       <c r="AD30" s="46" t="n">
         <v>2574</v>
@@ -3305,7 +3526,19 @@
         <v/>
       </c>
       <c r="Z31" s="28" t="n"/>
-      <c r="AA31" s="28" t="n"/>
+      <c r="AA31" s="28" t="inlineStr">
+        <is>
+          <t>binance_alpha</t>
+        </is>
+      </c>
+      <c r="AB31" t="n">
+        <v>47219.52</v>
+      </c>
+      <c r="AC31" t="inlineStr">
+        <is>
+          <t>ABSTAIN</t>
+        </is>
+      </c>
       <c r="AJ31" s="28">
         <f>IF(OR(AB31="",D31="",D31=0),"",AB31/D31)</f>
         <v/>
@@ -3318,37 +3551,37 @@
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="B32" t="n">
+      <c r="B32" s="28" t="n">
         <v>0.0010992966649597</v>
       </c>
-      <c r="C32">
+      <c r="C32" s="28">
         <f>IFERROR(B32/B31-1,"")</f>
         <v/>
       </c>
-      <c r="D32" t="n">
+      <c r="D32" s="28" t="n">
         <v>3484443.358583</v>
       </c>
-      <c r="E32" t="n">
+      <c r="E32" s="28" t="n">
         <v>0.4908091043332145</v>
       </c>
-      <c r="F32" t="n">
-        <v>5e-05</v>
-      </c>
-      <c r="G32" t="n">
-        <v>5e-05</v>
-      </c>
-      <c r="H32" t="n">
-        <v>5e-05</v>
-      </c>
-      <c r="I32" t="n">
+      <c r="F32" s="28" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="G32" s="28" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="H32" s="28" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="I32" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="J32" s="28" t="inlineStr">
         <is>
           <t>PINNED</t>
         </is>
       </c>
-      <c r="L32" t="n">
+      <c r="L32" s="28" t="n">
         <v>9658576.732218999</v>
       </c>
       <c r="O32" s="28" t="n">
@@ -3380,6 +3613,19 @@
         <f>IFERROR(P32/P29-1,"")</f>
         <v/>
       </c>
+      <c r="AA32" t="inlineStr">
+        <is>
+          <t>binance_alpha</t>
+        </is>
+      </c>
+      <c r="AB32" t="n">
+        <v>26797.74</v>
+      </c>
+      <c r="AC32" t="inlineStr">
+        <is>
+          <t>ABSTAIN</t>
+        </is>
+      </c>
       <c r="AJ32" s="28">
         <f>IF(OR(AB32="",D32="",D32=0),"",AB32/D32)</f>
         <v/>
@@ -3448,226 +3694,290 @@
         <f>IFERROR(P33/P30-1,"")</f>
         <v/>
       </c>
+      <c r="AA33" t="inlineStr">
+        <is>
+          <t>binance_alpha</t>
+        </is>
+      </c>
+      <c r="AB33" t="n">
+        <v>90721.38</v>
+      </c>
+      <c r="AC33" t="inlineStr">
+        <is>
+          <t>ABSTAIN</t>
+        </is>
+      </c>
       <c r="AJ33" s="28">
         <f>IF(OR(AB33="",D33="",D33=0),"",AB33/D33)</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="28" t="inlineStr">
         <is>
           <t>2026-08-01</t>
         </is>
       </c>
-      <c r="B34" t="n">
+      <c r="B34" s="28" t="n">
         <v>0.001387312420744</v>
       </c>
-      <c r="C34">
+      <c r="C34" s="28">
         <f>IFERROR(B34/B33-1,"")</f>
         <v/>
       </c>
-      <c r="D34" t="n">
+      <c r="D34" s="28" t="n">
         <v>14173987.853918</v>
       </c>
-      <c r="E34" t="n">
+      <c r="E34" s="28" t="n">
         <v>0.5132635677780482</v>
       </c>
-      <c r="F34" t="n">
+      <c r="F34" s="28" t="n">
         <v>0.0002554233333333</v>
       </c>
-      <c r="G34" t="n">
-        <v>5e-05</v>
-      </c>
-      <c r="H34" t="n">
+      <c r="G34" s="28" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="H34" s="28" t="n">
         <v>0.00056037</v>
       </c>
-      <c r="I34" t="n">
+      <c r="I34" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="L34" t="n">
+      <c r="L34" s="28" t="n">
         <v>12570735.627408</v>
       </c>
-      <c r="M34">
+      <c r="M34" s="28">
         <f>IFERROR(L34/MEDIAN(L20:L33),"")</f>
         <v/>
       </c>
-      <c r="O34" t="n">
+      <c r="O34" s="28" t="n">
         <v>1.5905</v>
       </c>
-      <c r="P34" t="n">
+      <c r="P34" s="28" t="n">
         <v>1.2753</v>
       </c>
-      <c r="Q34" t="n">
+      <c r="Q34" s="28" t="n">
         <v>1.6157</v>
       </c>
-      <c r="R34">
+      <c r="R34" s="28">
         <f>IFERROR(O34/P34,"")</f>
         <v/>
       </c>
-      <c r="S34">
+      <c r="S34" s="28">
         <f>IFERROR(AVERAGE(R32:R34),"")</f>
         <v/>
       </c>
-      <c r="T34">
+      <c r="T34" s="28">
         <f>IFERROR(Q34/Q29,"")</f>
         <v/>
       </c>
-      <c r="U34">
+      <c r="U34" s="28">
         <f>IFERROR(O34/O31-1,"")</f>
         <v/>
       </c>
-      <c r="V34">
+      <c r="V34" s="28">
         <f>IFERROR(P34/P31-1,"")</f>
         <v/>
       </c>
+      <c r="AA34" t="inlineStr">
+        <is>
+          <t>binance_alpha</t>
+        </is>
+      </c>
+      <c r="AB34" t="n">
+        <v>73042.56</v>
+      </c>
+      <c r="AC34" t="inlineStr">
+        <is>
+          <t>ABSTAIN</t>
+        </is>
+      </c>
+      <c r="AJ34">
+        <f>IF(OR(AB34="",AB34=0,D34="",D34=0),"",AB34/D34)</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="28" t="inlineStr">
         <is>
           <t>2026-08-02</t>
         </is>
       </c>
-      <c r="B35" t="n">
+      <c r="B35" s="28" t="n">
         <v>0.0013870979357402</v>
       </c>
-      <c r="C35">
+      <c r="C35" s="28">
         <f>IFERROR(B35/B34-1,"")</f>
         <v/>
       </c>
-      <c r="D35" t="n">
+      <c r="D35" s="28" t="n">
         <v>8050293.311166001</v>
       </c>
-      <c r="E35" t="n">
+      <c r="E35" s="28" t="n">
         <v>0.4690171507460309</v>
       </c>
-      <c r="F35" t="n">
+      <c r="F35" s="28" t="n">
         <v>0.000104545</v>
       </c>
-      <c r="G35" t="n">
-        <v>5e-05</v>
-      </c>
-      <c r="H35" t="n">
+      <c r="G35" s="28" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="H35" s="28" t="n">
         <v>0.00027156</v>
       </c>
-      <c r="I35" t="n">
+      <c r="I35" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="L35" t="n">
+      <c r="L35" s="28" t="n">
         <v>13201306.884897</v>
       </c>
-      <c r="M35">
+      <c r="M35" s="28">
         <f>IFERROR(L35/MEDIAN(L21:L34),"")</f>
         <v/>
       </c>
-      <c r="O35" t="n">
+      <c r="O35" s="28" t="n">
         <v>1.2863</v>
       </c>
-      <c r="P35" t="n">
+      <c r="P35" s="28" t="n">
         <v>1.5981</v>
       </c>
-      <c r="Q35" t="n">
+      <c r="Q35" s="28" t="n">
         <v>1.956</v>
       </c>
-      <c r="R35">
+      <c r="R35" s="28">
         <f>IFERROR(O35/P35,"")</f>
         <v/>
       </c>
-      <c r="S35">
+      <c r="S35" s="28">
         <f>IFERROR(AVERAGE(R33:R35),"")</f>
         <v/>
       </c>
-      <c r="T35">
+      <c r="T35" s="28">
         <f>IFERROR(Q35/Q30,"")</f>
         <v/>
       </c>
-      <c r="U35">
+      <c r="U35" s="28">
         <f>IFERROR(O35/O32-1,"")</f>
         <v/>
       </c>
-      <c r="V35">
+      <c r="V35" s="28">
         <f>IFERROR(P35/P32-1,"")</f>
         <v/>
       </c>
+      <c r="AA35" t="inlineStr">
+        <is>
+          <t>binance_alpha</t>
+        </is>
+      </c>
+      <c r="AB35" t="n">
+        <v>85610.19</v>
+      </c>
+      <c r="AC35" t="inlineStr">
+        <is>
+          <t>ABSTAIN</t>
+        </is>
+      </c>
+      <c r="AJ35">
+        <f>IF(OR(AB35="",AB35=0,D35="",D35=0),"",AB35/D35)</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="28" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="B36" t="n">
+      <c r="B36" s="28" t="n">
         <v>0.001259841794361022</v>
       </c>
-      <c r="C36">
+      <c r="C36" s="28">
         <f>IFERROR(B36/B35-1,"")</f>
         <v/>
       </c>
-      <c r="D36" t="n">
+      <c r="D36" s="28" t="n">
         <v>4779652.221457</v>
       </c>
-      <c r="E36" t="n">
+      <c r="E36" s="28" t="n">
         <v>0.4728796584260186</v>
       </c>
-      <c r="F36" t="n">
-        <v>5e-05</v>
-      </c>
-      <c r="G36" t="n">
-        <v>5e-05</v>
-      </c>
-      <c r="H36" t="n">
-        <v>5e-05</v>
-      </c>
-      <c r="I36" t="n">
+      <c r="F36" s="28" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="G36" s="28" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="H36" s="28" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="I36" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="J36" t="inlineStr">
+      <c r="J36" s="28" t="inlineStr">
         <is>
           <t>PINNED</t>
         </is>
       </c>
-      <c r="L36" t="n">
+      <c r="L36" s="28" t="n">
         <v>11828955.093356</v>
       </c>
-      <c r="M36">
+      <c r="M36" s="28">
         <f>IFERROR(L36/MEDIAN(L22:L35),"")</f>
         <v/>
       </c>
-      <c r="O36" t="n">
+      <c r="O36" s="28" t="n">
         <v>1.3504</v>
       </c>
-      <c r="P36" t="n">
+      <c r="P36" s="28" t="n">
         <v>1.7367</v>
       </c>
-      <c r="Q36" t="n">
+      <c r="Q36" s="28" t="n">
         <v>2.0665</v>
       </c>
-      <c r="R36">
+      <c r="R36" s="28">
         <f>IFERROR(O36/P36,"")</f>
         <v/>
       </c>
-      <c r="S36">
+      <c r="S36" s="28">
         <f>IFERROR(AVERAGE(R34:R36),"")</f>
         <v/>
       </c>
-      <c r="T36">
+      <c r="T36" s="28">
         <f>IFERROR(Q36/Q31,"")</f>
         <v/>
       </c>
-      <c r="U36">
+      <c r="U36" s="28">
         <f>IFERROR(O36/O33-1,"")</f>
         <v/>
       </c>
-      <c r="V36">
+      <c r="V36" s="28">
         <f>IFERROR(P36/P33-1,"")</f>
+        <v/>
+      </c>
+      <c r="AA36" t="inlineStr">
+        <is>
+          <t>binance_alpha</t>
+        </is>
+      </c>
+      <c r="AB36" t="n">
+        <v>66713.63</v>
+      </c>
+      <c r="AC36" t="inlineStr">
+        <is>
+          <t>ABSTAIN</t>
+        </is>
+      </c>
+      <c r="AJ36">
+        <f>IF(OR(AB36="",AB36=0,D36="",D36=0),"",AB36/D36)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A1:Z1"/>
+    <mergeCell ref="AA1:AJ1"/>
     <mergeCell ref="AK1:AM1"/>
-    <mergeCell ref="A1:Z1"/>
     <mergeCell ref="AN1:AO1"/>
-    <mergeCell ref="AA1:AJ1"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>